<commit_message>
Updated Test 6 : signup page test and added check your mail page validation after clicking submit on sign up page
</commit_message>
<xml_diff>
--- a/TestData/ExcelFiles/Test Data1.xlsx
+++ b/TestData/ExcelFiles/Test Data1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AutomationTraining\CreatioCRM\TestData\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26976F3B-CF3D-42EF-A87A-B571ADB99958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B205423-92C4-46DA-B24C-F31675FBABC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4920" yWindow="504" windowWidth="10596" windowHeight="10740" firstSheet="2" activeTab="2" xr2:uid="{71A6E62E-4B9F-4364-B2A5-18FEFE15415A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{71A6E62E-4B9F-4364-B2A5-18FEFE15415A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="54">
   <si>
     <t>Url</t>
   </si>
@@ -186,6 +186,9 @@
   </si>
   <si>
     <t>somanjan1606Invalid@gmail.com</t>
+  </si>
+  <si>
+    <t>Sp@369stark</t>
   </si>
 </sst>
 </file>
@@ -817,7 +820,7 @@
         <v>49</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -841,6 +844,7 @@
     <hyperlink ref="A2" r:id="rId1" xr:uid="{A86A69B9-F383-4C53-8582-29ABCB8B323B}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{1B7A8B6A-D536-408F-B7BF-0282847AD0EF}"/>
     <hyperlink ref="A4" r:id="rId3" xr:uid="{FF337F46-27CF-4F08-A501-F3C64B8026F1}"/>
+    <hyperlink ref="B2" r:id="rId4" xr:uid="{EE0A992F-4021-4EA2-AE2E-CD5EB386E840}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated test cases : seperate test cases for valid and invalid login credential and also added few more verification for signUp page and invalid login credential
</commit_message>
<xml_diff>
--- a/TestData/ExcelFiles/Test Data1.xlsx
+++ b/TestData/ExcelFiles/Test Data1.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AutomationTraining\CreatioCRM\TestData\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B205423-92C4-46DA-B24C-F31675FBABC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2EA500-F099-4CB4-956E-47B0BD3DD06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{71A6E62E-4B9F-4364-B2A5-18FEFE15415A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="2" activeTab="2" xr2:uid="{71A6E62E-4B9F-4364-B2A5-18FEFE15415A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="verifyApplicationSignUp" sheetId="2" r:id="rId2"/>
-    <sheet name="verifyApplicationLogin" sheetId="3" r:id="rId3"/>
+    <sheet name="verifySuccessulApplicationLogin" sheetId="3" r:id="rId3"/>
+    <sheet name="verifyInvalidApplicationLogin" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
   <si>
     <t>Url</t>
   </si>
@@ -195,7 +196,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -236,6 +237,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -264,7 +280,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -274,6 +290,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -800,7 +819,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B9DDEE3-C0EF-414A-AB36-FAF8E8F794B8}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -823,28 +842,48 @@
         <v>53</v>
       </c>
     </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A11987B-5002-4F41-95EE-E700A05168F3}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="B3" s="7" t="s">
         <v>50</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{A86A69B9-F383-4C53-8582-29ABCB8B323B}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{1B7A8B6A-D536-408F-B7BF-0282847AD0EF}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{FF337F46-27CF-4F08-A501-F3C64B8026F1}"/>
-    <hyperlink ref="B2" r:id="rId4" xr:uid="{EE0A992F-4021-4EA2-AE2E-CD5EB386E840}"/>
+    <hyperlink ref="A2" r:id="rId1" display="mailto:somanjan1606Invalid@gmail.com" xr:uid="{A3A82A45-40DB-4C7C-8E11-926D81B0908A}"/>
+    <hyperlink ref="A3" r:id="rId2" display="mailto:somanjan1606Invalid@gmail.com" xr:uid="{0B671351-6421-40B5-99E6-E1B4BA609302}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>